<commit_message>
fix(import): undo large batches and show cancelled batch page
- undo_import_batch (new migration, same rules and deletions): counts all
  blockers instead of listing only 50, groups them by cause (the import
  that added them, or changes by hand) and gives each one its party.
- Blocked undo view: what caused it, with a link to the other import and
  what to do; parties involved with links, the first 20 and the rest
  behind "Mostra". Scrolled into view.
- The page of a cancelled import shows "Import annullato il …" with the
  counts saved on the batch and reads no deleted rows.
- The undo result is parsed into strings and numbers only (lib/import/undo);
  the action logs durations and counts.
- Fixture IDs moved to the 90000 range: real imports on staging used some
  of the old ones. SQL test for a large batch blocked by a second import.
</commit_message>
<xml_diff>
--- a/tests/fixtures/crm-parcheggio-2026-finto.xlsx
+++ b/tests/fixtures/crm-parcheggio-2026-finto.xlsx
@@ -1743,7 +1743,7 @@
         <v>15</v>
       </c>
       <c r="B2" s="1">
-        <v>73</v>
+        <v>90073</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>16</v>
@@ -1799,7 +1799,7 @@
         <v>25</v>
       </c>
       <c r="B3" s="1">
-        <v>301</v>
+        <v>90301</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>26</v>
@@ -1849,7 +1849,7 @@
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1">
-        <v>659</v>
+        <v>90659</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>35</v>
@@ -1891,7 +1891,7 @@
         <v>41</v>
       </c>
       <c r="B5" s="1">
-        <v>660</v>
+        <v>90660</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>42</v>
@@ -1965,7 +1965,7 @@
     <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1">
-        <v>700</v>
+        <v>90700</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>51</v>
@@ -2001,7 +2001,7 @@
         <v>25</v>
       </c>
       <c r="B8" s="1">
-        <v>701</v>
+        <v>90701</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>54</v>
@@ -2049,7 +2049,7 @@
     <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="1">
-        <v>702</v>
+        <v>90702</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>62</v>
@@ -2083,7 +2083,7 @@
     <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="1">
-        <v>703</v>
+        <v>90703</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>65</v>
@@ -2117,7 +2117,7 @@
         <v>41</v>
       </c>
       <c r="B11" s="1">
-        <v>704</v>
+        <v>90704</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>67</v>
@@ -2159,7 +2159,7 @@
         <v>25</v>
       </c>
       <c r="B12" s="1">
-        <v>705</v>
+        <v>90705</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>72</v>
@@ -2203,7 +2203,7 @@
         <v>15</v>
       </c>
       <c r="B13" s="1">
-        <v>1200</v>
+        <v>91200</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>78</v>
@@ -2255,7 +2255,7 @@
     <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="1">
-        <v>2000</v>
+        <v>92000</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>86</v>
@@ -2307,7 +2307,7 @@
         <v>41</v>
       </c>
       <c r="B15" s="1">
-        <v>2001</v>
+        <v>92001</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>92</v>
@@ -2351,7 +2351,7 @@
         <v>25</v>
       </c>
       <c r="B16" s="1">
-        <v>2002</v>
+        <v>92002</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>97</v>
@@ -2399,7 +2399,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="1">
-        <v>2003</v>
+        <v>92003</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>102</v>
@@ -2445,7 +2445,7 @@
     <row r="18" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="1">
-        <v>2004</v>
+        <v>92004</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>109</v>
@@ -2491,7 +2491,7 @@
         <v>41</v>
       </c>
       <c r="B19" s="1">
-        <v>2005</v>
+        <v>92005</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>115</v>
@@ -2537,7 +2537,7 @@
         <v>25</v>
       </c>
       <c r="B20" s="1">
-        <v>2006</v>
+        <v>92006</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>119</v>
@@ -2589,7 +2589,7 @@
         <v>15</v>
       </c>
       <c r="B21" s="1">
-        <v>2007</v>
+        <v>92007</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>126</v>
@@ -2631,7 +2631,7 @@
     <row r="22" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="1">
-        <v>2008</v>
+        <v>92008</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>131</v>
@@ -2677,7 +2677,7 @@
         <v>41</v>
       </c>
       <c r="B23" s="1">
-        <v>2009</v>
+        <v>92009</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>137</v>
@@ -2725,7 +2725,7 @@
         <v>25</v>
       </c>
       <c r="B24" s="1">
-        <v>2010</v>
+        <v>92010</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>143</v>
@@ -2775,7 +2775,7 @@
         <v>15</v>
       </c>
       <c r="B25" s="1">
-        <v>2011</v>
+        <v>92011</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>148</v>
@@ -2817,7 +2817,7 @@
     <row r="26" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="1">
-        <v>2012</v>
+        <v>92012</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>152</v>
@@ -2867,7 +2867,7 @@
         <v>41</v>
       </c>
       <c r="B27" s="1">
-        <v>2013</v>
+        <v>92013</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>156</v>
@@ -2911,7 +2911,7 @@
         <v>25</v>
       </c>
       <c r="B28" s="1">
-        <v>2014</v>
+        <v>92014</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>160</v>
@@ -2959,7 +2959,7 @@
         <v>15</v>
       </c>
       <c r="B29" s="1">
-        <v>2015</v>
+        <v>92015</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>165</v>
@@ -3007,7 +3007,7 @@
     <row r="30" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="1">
-        <v>2016</v>
+        <v>92016</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>169</v>
@@ -3053,7 +3053,7 @@
         <v>41</v>
       </c>
       <c r="B31" s="1">
-        <v>2017</v>
+        <v>92017</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>173</v>
@@ -3097,7 +3097,7 @@
         <v>25</v>
       </c>
       <c r="B32" s="1">
-        <v>2018</v>
+        <v>92018</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>177</v>
@@ -3149,7 +3149,7 @@
         <v>15</v>
       </c>
       <c r="B33" s="1">
-        <v>2019</v>
+        <v>92019</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>182</v>
@@ -3191,7 +3191,7 @@
     <row r="34" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="1">
-        <v>2020</v>
+        <v>92020</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>186</v>
@@ -3239,7 +3239,7 @@
         <v>41</v>
       </c>
       <c r="B35" s="1">
-        <v>2021</v>
+        <v>92021</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>190</v>
@@ -3287,7 +3287,7 @@
         <v>25</v>
       </c>
       <c r="B36" s="1">
-        <v>2022</v>
+        <v>92022</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>194</v>
@@ -3335,7 +3335,7 @@
         <v>15</v>
       </c>
       <c r="B37" s="1">
-        <v>2023</v>
+        <v>92023</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>199</v>
@@ -3377,7 +3377,7 @@
     <row r="38" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="1">
-        <v>2024</v>
+        <v>92024</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>203</v>
@@ -3427,7 +3427,7 @@
         <v>41</v>
       </c>
       <c r="B39" s="1">
-        <v>2025</v>
+        <v>92025</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>207</v>
@@ -3473,7 +3473,7 @@
         <v>25</v>
       </c>
       <c r="B40" s="1">
-        <v>2026</v>
+        <v>92026</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>211</v>
@@ -3521,7 +3521,7 @@
         <v>15</v>
       </c>
       <c r="B41" s="1">
-        <v>2027</v>
+        <v>92027</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>216</v>
@@ -3567,7 +3567,7 @@
     <row r="42" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
       <c r="B42" s="1">
-        <v>2028</v>
+        <v>92028</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>220</v>
@@ -3613,7 +3613,7 @@
         <v>41</v>
       </c>
       <c r="B43" s="1">
-        <v>2029</v>
+        <v>92029</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>224</v>
@@ -3657,7 +3657,7 @@
         <v>25</v>
       </c>
       <c r="B44" s="1">
-        <v>2030</v>
+        <v>92030</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>228</v>
@@ -3711,7 +3711,7 @@
         <v>15</v>
       </c>
       <c r="B45" s="1">
-        <v>2031</v>
+        <v>92031</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>233</v>
@@ -3753,7 +3753,7 @@
     <row r="46" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="1">
-        <v>2032</v>
+        <v>92032</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>237</v>
@@ -3799,7 +3799,7 @@
         <v>41</v>
       </c>
       <c r="B47" s="1">
-        <v>2033</v>
+        <v>92033</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>241</v>
@@ -3847,7 +3847,7 @@
         <v>25</v>
       </c>
       <c r="B48" s="1">
-        <v>2034</v>
+        <v>92034</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>245</v>
@@ -3895,7 +3895,7 @@
         <v>15</v>
       </c>
       <c r="B49" s="1">
-        <v>2035</v>
+        <v>92035</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>250</v>
@@ -3939,7 +3939,7 @@
     <row r="50" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
       <c r="B50" s="1">
-        <v>2036</v>
+        <v>92036</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>254</v>
@@ -3989,7 +3989,7 @@
         <v>41</v>
       </c>
       <c r="B51" s="1">
-        <v>2037</v>
+        <v>92037</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>258</v>
@@ -4033,7 +4033,7 @@
         <v>25</v>
       </c>
       <c r="B52" s="1">
-        <v>2038</v>
+        <v>92038</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>262</v>
@@ -4081,7 +4081,7 @@
         <v>15</v>
       </c>
       <c r="B53" s="1">
-        <v>2039</v>
+        <v>92039</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>266</v>
@@ -4127,7 +4127,7 @@
     <row r="54" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A54" s="1"/>
       <c r="B54" s="1">
-        <v>2040</v>
+        <v>92040</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>270</v>
@@ -4175,7 +4175,7 @@
         <v>41</v>
       </c>
       <c r="B55" s="1">
-        <v>2041</v>
+        <v>92041</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>274</v>
@@ -4219,7 +4219,7 @@
         <v>25</v>
       </c>
       <c r="B56" s="1">
-        <v>2042</v>
+        <v>92042</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>278</v>
@@ -4271,7 +4271,7 @@
         <v>15</v>
       </c>
       <c r="B57" s="1">
-        <v>2043</v>
+        <v>92043</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>282</v>
@@ -4313,7 +4313,7 @@
     <row r="58" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A58" s="1"/>
       <c r="B58" s="1">
-        <v>2044</v>
+        <v>92044</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>286</v>
@@ -4359,7 +4359,7 @@
         <v>41</v>
       </c>
       <c r="B59" s="1">
-        <v>2045</v>
+        <v>92045</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>290</v>
@@ -4409,7 +4409,7 @@
         <v>25</v>
       </c>
       <c r="B60" s="1">
-        <v>2046</v>
+        <v>92046</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>294</v>
@@ -4457,7 +4457,7 @@
         <v>15</v>
       </c>
       <c r="B61" s="1">
-        <v>2047</v>
+        <v>92047</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>298</v>
@@ -4499,7 +4499,7 @@
     <row r="62" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
       <c r="B62" s="1">
-        <v>2048</v>
+        <v>92048</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>302</v>
@@ -4549,7 +4549,7 @@
         <v>41</v>
       </c>
       <c r="B63" s="1">
-        <v>2049</v>
+        <v>92049</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>306</v>
@@ -4593,7 +4593,7 @@
         <v>25</v>
       </c>
       <c r="B64" s="1">
-        <v>2050</v>
+        <v>92050</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>310</v>
@@ -4643,7 +4643,7 @@
         <v>15</v>
       </c>
       <c r="B65" s="1">
-        <v>2051</v>
+        <v>92051</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>314</v>
@@ -4689,7 +4689,7 @@
     <row r="66" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A66" s="1"/>
       <c r="B66" s="1">
-        <v>2052</v>
+        <v>92052</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>318</v>
@@ -4735,7 +4735,7 @@
         <v>41</v>
       </c>
       <c r="B67" s="1">
-        <v>2053</v>
+        <v>92053</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>322</v>
@@ -4777,7 +4777,7 @@
         <v>25</v>
       </c>
       <c r="B68" s="1">
-        <v>2054</v>
+        <v>92054</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>325</v>
@@ -4827,7 +4827,7 @@
         <v>15</v>
       </c>
       <c r="B69" s="1">
-        <v>2055</v>
+        <v>92055</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>328</v>
@@ -4869,7 +4869,7 @@
     <row r="70" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A70" s="1"/>
       <c r="B70" s="1">
-        <v>2056</v>
+        <v>92056</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>331</v>
@@ -4913,7 +4913,7 @@
         <v>41</v>
       </c>
       <c r="B71" s="1">
-        <v>2057</v>
+        <v>92057</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>334</v>
@@ -4959,7 +4959,7 @@
         <v>25</v>
       </c>
       <c r="B72" s="1">
-        <v>2058</v>
+        <v>92058</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>337</v>
@@ -5005,7 +5005,7 @@
         <v>15</v>
       </c>
       <c r="B73" s="1">
-        <v>2059</v>
+        <v>92059</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>340</v>
@@ -5045,7 +5045,7 @@
     <row r="74" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A74" s="1"/>
       <c r="B74" s="1">
-        <v>2060</v>
+        <v>92060</v>
       </c>
       <c r="C74" s="1" t="s">
         <v>343</v>
@@ -5095,7 +5095,7 @@
         <v>41</v>
       </c>
       <c r="B75" s="1">
-        <v>2061</v>
+        <v>92061</v>
       </c>
       <c r="C75" s="1" t="s">
         <v>346</v>
@@ -5137,7 +5137,7 @@
         <v>25</v>
       </c>
       <c r="B76" s="1">
-        <v>2062</v>
+        <v>92062</v>
       </c>
       <c r="C76" s="1" t="s">
         <v>349</v>
@@ -5183,7 +5183,7 @@
         <v>15</v>
       </c>
       <c r="B77" s="1">
-        <v>2063</v>
+        <v>92063</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>352</v>
@@ -5227,7 +5227,7 @@
     <row r="78" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A78" s="1"/>
       <c r="B78" s="1">
-        <v>2064</v>
+        <v>92064</v>
       </c>
       <c r="C78" s="1" t="s">
         <v>355</v>
@@ -5271,7 +5271,7 @@
         <v>41</v>
       </c>
       <c r="B79" s="1">
-        <v>2065</v>
+        <v>92065</v>
       </c>
       <c r="C79" s="1" t="s">
         <v>358</v>
@@ -5315,7 +5315,7 @@
         <v>25</v>
       </c>
       <c r="B80" s="1">
-        <v>2066</v>
+        <v>92066</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>361</v>
@@ -5365,7 +5365,7 @@
         <v>15</v>
       </c>
       <c r="B81" s="1">
-        <v>2067</v>
+        <v>92067</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>364</v>
@@ -5405,7 +5405,7 @@
     <row r="82" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A82" s="1"/>
       <c r="B82" s="1">
-        <v>2068</v>
+        <v>92068</v>
       </c>
       <c r="C82" s="1" t="s">
         <v>367</v>
@@ -5449,7 +5449,7 @@
         <v>41</v>
       </c>
       <c r="B83" s="1">
-        <v>2069</v>
+        <v>92069</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>370</v>
@@ -5495,7 +5495,7 @@
         <v>25</v>
       </c>
       <c r="B84" s="1">
-        <v>2070</v>
+        <v>92070</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>373</v>
@@ -5543,7 +5543,7 @@
         <v>15</v>
       </c>
       <c r="B85" s="1">
-        <v>2071</v>
+        <v>92071</v>
       </c>
       <c r="C85" s="1" t="s">
         <v>376</v>

</xml_diff>